<commit_message>
subir listados campaña corazul5
</commit_message>
<xml_diff>
--- a/campanas/260413_corazul/corazul_1_tuesday.xlsx
+++ b/campanas/260413_corazul/corazul_1_tuesday.xlsx
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diegopaezmacias/Library/Mobile Documents/com~apple~CloudDocs/GRIDDED.AGENCY/PROYECTOS/2026/02 MIRAMAR CRUISES/Agente Descubierta/03 Campañas agente descubierta/260407 Corazul/listado envios/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diegopaezmacias/GRIDDED.AGENCY local/00_GRIDDED AGENCY/cdn/campanas/260413_corazul/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D82B77FB-B274-6440-98BF-82FCEC473BD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1769A763-E529-0341-B6F3-BF6D58E3EB9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="44800" windowHeight="24600" xr2:uid="{FE8E41CE-C1E5-794B-8212-B8E3CEE34DA9}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="19560" windowHeight="24600" xr2:uid="{FE8E41CE-C1E5-794B-8212-B8E3CEE34DA9}"/>
   </bookViews>
   <sheets>
     <sheet name="campaña 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="DatosExternos_2" localSheetId="0" hidden="1">'campaña 1'!$A$1:$H$51</definedName>
+    <definedName name="DatosExternos_2" localSheetId="0" hidden="1">'campaña 1'!$A$1:$H$50</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="304">
   <si>
     <t>nombreNaviera</t>
   </si>
@@ -73,15 +73,6 @@
   </si>
   <si>
     <t>Costa Cruceros</t>
-  </si>
-  <si>
-    <t>DIEGO</t>
-  </si>
-  <si>
-    <t>PAEZ</t>
-  </si>
-  <si>
-    <t>A CORUÑA</t>
   </si>
   <si>
     <t>GEMMA</t>
@@ -1072,8 +1063,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EBC5DAF2-265F-5C4B-9F14-50406A6420A0}" name="Ventas_Cuadruples_2025" displayName="Ventas_Cuadruples_2025" ref="A1:H51" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:H51" xr:uid="{7B6879F4-F5E9-40D9-A981-23B705F0A713}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EBC5DAF2-265F-5C4B-9F14-50406A6420A0}" name="Ventas_Cuadruples_2025" displayName="Ventas_Cuadruples_2025" ref="A1:H50" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:H50" xr:uid="{7B6879F4-F5E9-40D9-A981-23B705F0A713}"/>
   <tableColumns count="8">
     <tableColumn id="2" xr3:uid="{D7C59A67-56B1-FC40-A80E-0553C9334F80}" uniqueName="2" name="nombreNaviera" queryTableFieldId="2" dataDxfId="7"/>
     <tableColumn id="3" xr3:uid="{B6B681FD-4C35-654A-AEF6-F0A60C2EF737}" uniqueName="3" name="nombreCliente" queryTableFieldId="3" dataDxfId="6"/>
@@ -1385,7 +1376,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E88A72D-71A2-D844-BACB-214CA146513D}">
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
@@ -1436,427 +1427,436 @@
       <c r="C2" t="s">
         <v>10</v>
       </c>
-      <c r="D2">
-        <v>609508399</v>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>13</v>
       </c>
       <c r="G2" t="s">
-        <v>11</v>
+        <v>14</v>
+      </c>
+      <c r="H2" s="1">
+        <v>45900</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E3" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F3" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G3" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="H3" s="1">
-        <v>45900</v>
+        <v>45829</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G4" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="H4" s="1">
-        <v>45829</v>
+        <v>45837</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="G5" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="H5" s="1">
-        <v>45837</v>
+        <v>45776</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E6" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="F6" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="G6" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="H6" s="1">
-        <v>45776</v>
+        <v>45793</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C7" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D7" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="E7" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F7" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="G7" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="H7" s="1">
-        <v>45793</v>
+        <v>45829</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C8" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E8" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F8" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G8" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="H8" s="1">
-        <v>45829</v>
+        <v>45702</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C9" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D9" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="E9" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F9" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="G9" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H9" s="1">
-        <v>45702</v>
+        <v>45717</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C10" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D10" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E10" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="F10" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="H10" s="1">
-        <v>45717</v>
+        <v>45975</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C11" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D11" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E11" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F11" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="G11" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="H11" s="1">
-        <v>45975</v>
+        <v>45768</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B12" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C12" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D12" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E12" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="F12" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="G12" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="H12" s="1">
-        <v>45768</v>
+        <v>46013</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C13" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D13" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E13" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="F13" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="G13" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="H13" s="1">
-        <v>46013</v>
+        <v>45722</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C14" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D14" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="E14" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="F14" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="G14" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="H14" s="1">
-        <v>45722</v>
+        <v>45869</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B15" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C15" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D15" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="E15" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="F15" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="G15" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H15" s="1">
-        <v>45869</v>
+        <v>45862</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C16" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D16" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E16" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="F16" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="G16" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="H16" s="1">
-        <v>45862</v>
+        <v>45829</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>18</v>
+        <v>100</v>
       </c>
       <c r="B17" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C17" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D17" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="E17" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="F17" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="G17" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="H17" s="1">
-        <v>45829</v>
+        <v>45900</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>103</v>
+        <v>8</v>
       </c>
       <c r="B18" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C18" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D18" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="E18" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="F18" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="G18" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="H18" s="1">
-        <v>45900</v>
+        <v>45823</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
@@ -1864,129 +1864,129 @@
         <v>8</v>
       </c>
       <c r="B19" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C19" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D19" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="E19" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="F19" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="G19" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="H19" s="1">
-        <v>45823</v>
+        <v>45859</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>8</v>
+        <v>119</v>
       </c>
       <c r="B20" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C20" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D20" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E20" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F20" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G20" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="H20" s="1">
-        <v>45859</v>
+        <v>45892</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>122</v>
+        <v>8</v>
       </c>
       <c r="B21" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C21" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D21" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="E21" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="F21" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="G21" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="H21" s="1">
-        <v>45892</v>
+        <v>45773</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B22" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="C22" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="D22" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="E22" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="F22" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="G22" t="s">
-        <v>134</v>
+        <v>39</v>
       </c>
       <c r="H22" s="1">
-        <v>45773</v>
+        <v>45827</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B23" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C23" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D23" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E23" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F23" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G23" t="s">
-        <v>42</v>
+        <v>142</v>
       </c>
       <c r="H23" s="1">
-        <v>45827</v>
+        <v>45887</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
@@ -1994,155 +1994,155 @@
         <v>8</v>
       </c>
       <c r="B24" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C24" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D24" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="E24" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="F24" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="G24" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="H24" s="1">
-        <v>45887</v>
+        <v>45781</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B25" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C25" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="D25" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="E25" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="F25" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="G25" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="H25" s="1">
-        <v>45781</v>
+        <v>45829</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B26" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="C26" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="D26" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="E26" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="F26" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="G26" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="H26" s="1">
-        <v>45829</v>
+        <v>45724</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B27" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C27" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="D27" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="E27" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="F27" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="G27" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="H27" s="1">
-        <v>45724</v>
+        <v>45921</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>8</v>
+        <v>167</v>
       </c>
       <c r="B28" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C28" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="D28" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="E28" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="F28" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="G28" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="H28" s="1">
-        <v>45921</v>
+        <v>45870</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>170</v>
+        <v>8</v>
       </c>
       <c r="B29" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="C29" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="D29" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="E29" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="F29" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="G29" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="H29" s="1">
-        <v>45870</v>
+        <v>45767</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
@@ -2150,441 +2150,441 @@
         <v>8</v>
       </c>
       <c r="B30" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C30" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D30" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="E30" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="F30" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="G30" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="H30" s="1">
-        <v>45767</v>
+        <v>45844</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B31" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="C31" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D31" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E31" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="F31" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="G31" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="H31" s="1">
-        <v>45844</v>
+        <v>45841</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B32" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C32" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="D32" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="E32" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="F32" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="G32" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="H32" s="1">
-        <v>45841</v>
+        <v>45955</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B33" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="C33" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="D33" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="E33" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="F33" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="G33" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="H33" s="1">
-        <v>45955</v>
+        <v>45864</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B34" t="s">
-        <v>201</v>
+        <v>174</v>
       </c>
       <c r="C34" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="D34" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E34" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F34" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="G34" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="H34" s="1">
-        <v>45864</v>
+        <v>45801</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B35" t="s">
-        <v>177</v>
+        <v>209</v>
       </c>
       <c r="C35" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D35" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E35" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="F35" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="G35" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="H35" s="1">
-        <v>45801</v>
+        <v>45815</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B36" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="C36" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="D36" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="E36" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F36" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="G36" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="H36" s="1">
-        <v>45815</v>
+        <v>45773</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B37" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="C37" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="D37" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="E37" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="F37" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="G37" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="H37" s="1">
-        <v>45773</v>
+        <v>45871</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B38" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="C38" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="D38" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="E38" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="F38" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="G38" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="H38" s="1">
-        <v>45871</v>
+        <v>45886</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B39" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="C39" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="D39" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="E39" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="F39" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="G39" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="H39" s="1">
-        <v>45886</v>
+        <v>45781</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B40" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C40" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="D40" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="E40" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="F40" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="G40" t="s">
-        <v>241</v>
+        <v>160</v>
       </c>
       <c r="H40" s="1">
-        <v>45781</v>
+        <v>45821</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B41" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C41" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D41" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="E41" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="F41" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="G41" t="s">
-        <v>163</v>
+        <v>249</v>
       </c>
       <c r="H41" s="1">
-        <v>45821</v>
+        <v>45856</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B42" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="C42" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="D42" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="E42" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="F42" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="G42" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="H42" s="1">
-        <v>45856</v>
+        <v>45899</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B43" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="C43" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="D43" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="E43" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="F43" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="G43" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="H43" s="1">
-        <v>45899</v>
+        <v>45873</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B44" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="C44" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="D44" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="E44" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="F44" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="G44" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="H44" s="1">
-        <v>45873</v>
+        <v>45827</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B45" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="C45" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="D45" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="E45" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="F45" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="G45" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="H45" s="1">
-        <v>45827</v>
+        <v>45849</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B46" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="C46" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="D46" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="E46" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="F46" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="G46" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="H46" s="1">
-        <v>45849</v>
+        <v>45851</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
@@ -2592,25 +2592,25 @@
         <v>8</v>
       </c>
       <c r="B47" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="C47" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="D47" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="E47" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="F47" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="G47" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="H47" s="1">
-        <v>45851</v>
+        <v>45961</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
@@ -2618,25 +2618,25 @@
         <v>8</v>
       </c>
       <c r="B48" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="C48" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="D48" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="E48" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="F48" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="G48" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="H48" s="1">
-        <v>45961</v>
+        <v>45844</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
@@ -2644,25 +2644,25 @@
         <v>8</v>
       </c>
       <c r="B49" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="C49" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="D49" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="E49" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="F49" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="G49" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="H49" s="1">
-        <v>45844</v>
+        <v>45804</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.2">
@@ -2670,50 +2670,24 @@
         <v>8</v>
       </c>
       <c r="B50" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="C50" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="D50" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="E50" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="F50" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="G50" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="H50" s="1">
-        <v>45804</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
-        <v>8</v>
-      </c>
-      <c r="B51" t="s">
-        <v>301</v>
-      </c>
-      <c r="C51" t="s">
-        <v>302</v>
-      </c>
-      <c r="D51" t="s">
-        <v>303</v>
-      </c>
-      <c r="E51" t="s">
-        <v>304</v>
-      </c>
-      <c r="F51" t="s">
-        <v>305</v>
-      </c>
-      <c r="G51" t="s">
-        <v>306</v>
-      </c>
-      <c r="H51" s="1">
         <v>45874</v>
       </c>
     </row>

</xml_diff>

<commit_message>
subir listados campaña corazul6
</commit_message>
<xml_diff>
--- a/campanas/260413_corazul/corazul_1_tuesday.xlsx
+++ b/campanas/260413_corazul/corazul_1_tuesday.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diegopaezmacias/GRIDDED.AGENCY local/00_GRIDDED AGENCY/cdn/campanas/260413_corazul/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1769A763-E529-0341-B6F3-BF6D58E3EB9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A302FD52-50A0-9043-A6D2-012873BA9B3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="19560" windowHeight="24600" xr2:uid="{FE8E41CE-C1E5-794B-8212-B8E3CEE34DA9}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="campaña 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="DatosExternos_2" localSheetId="0" hidden="1">'campaña 1'!$A$1:$H$50</definedName>
+    <definedName name="DatosExternos_2" localSheetId="0" hidden="1">'campaña 1'!$A$1:$H$49</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="304">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="298">
   <si>
     <t>nombreNaviera</t>
   </si>
@@ -73,24 +73,6 @@
   </si>
   <si>
     <t>Costa Cruceros</t>
-  </si>
-  <si>
-    <t>GEMMA</t>
-  </si>
-  <si>
-    <t>DEL MORAL MONGE</t>
-  </si>
-  <si>
-    <t>+34661622876</t>
-  </si>
-  <si>
-    <t>gemadelmoralmonge@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PL DOñA ELADIA Nº 3 </t>
-  </si>
-  <si>
-    <t>MARCHAMALO</t>
   </si>
   <si>
     <t>MSC Cruceros</t>
@@ -1063,8 +1045,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EBC5DAF2-265F-5C4B-9F14-50406A6420A0}" name="Ventas_Cuadruples_2025" displayName="Ventas_Cuadruples_2025" ref="A1:H50" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:H50" xr:uid="{7B6879F4-F5E9-40D9-A981-23B705F0A713}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EBC5DAF2-265F-5C4B-9F14-50406A6420A0}" name="Ventas_Cuadruples_2025" displayName="Ventas_Cuadruples_2025" ref="A1:H49" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:H49" xr:uid="{7B6879F4-F5E9-40D9-A981-23B705F0A713}"/>
   <tableColumns count="8">
     <tableColumn id="2" xr3:uid="{D7C59A67-56B1-FC40-A80E-0553C9334F80}" uniqueName="2" name="nombreNaviera" queryTableFieldId="2" dataDxfId="7"/>
     <tableColumn id="3" xr3:uid="{B6B681FD-4C35-654A-AEF6-F0A60C2EF737}" uniqueName="3" name="nombreCliente" queryTableFieldId="3" dataDxfId="6"/>
@@ -1376,7 +1358,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E88A72D-71A2-D844-BACB-214CA146513D}">
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
@@ -1419,33 +1401,33 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H2" s="1">
-        <v>45900</v>
+        <v>45829</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
         <v>16</v>
@@ -1466,12 +1448,12 @@
         <v>21</v>
       </c>
       <c r="H3" s="1">
-        <v>45829</v>
+        <v>45837</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
         <v>22</v>
@@ -1492,12 +1474,12 @@
         <v>27</v>
       </c>
       <c r="H4" s="1">
-        <v>45837</v>
+        <v>45776</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
         <v>28</v>
@@ -1518,12 +1500,12 @@
         <v>33</v>
       </c>
       <c r="H5" s="1">
-        <v>45776</v>
+        <v>45793</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
         <v>34</v>
@@ -1544,12 +1526,12 @@
         <v>39</v>
       </c>
       <c r="H6" s="1">
-        <v>45793</v>
+        <v>45829</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B7" t="s">
         <v>40</v>
@@ -1570,12 +1552,12 @@
         <v>45</v>
       </c>
       <c r="H7" s="1">
-        <v>45829</v>
+        <v>45702</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B8" t="s">
         <v>46</v>
@@ -1596,12 +1578,12 @@
         <v>51</v>
       </c>
       <c r="H8" s="1">
-        <v>45702</v>
+        <v>45717</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B9" t="s">
         <v>52</v>
@@ -1622,12 +1604,12 @@
         <v>57</v>
       </c>
       <c r="H9" s="1">
-        <v>45717</v>
+        <v>45975</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B10" t="s">
         <v>58</v>
@@ -1648,12 +1630,12 @@
         <v>63</v>
       </c>
       <c r="H10" s="1">
-        <v>45975</v>
+        <v>45768</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B11" t="s">
         <v>64</v>
@@ -1674,12 +1656,12 @@
         <v>69</v>
       </c>
       <c r="H11" s="1">
-        <v>45768</v>
+        <v>46013</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B12" t="s">
         <v>70</v>
@@ -1700,12 +1682,12 @@
         <v>75</v>
       </c>
       <c r="H12" s="1">
-        <v>46013</v>
+        <v>45722</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B13" t="s">
         <v>76</v>
@@ -1726,12 +1708,12 @@
         <v>81</v>
       </c>
       <c r="H13" s="1">
-        <v>45722</v>
+        <v>45869</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B14" t="s">
         <v>82</v>
@@ -1752,12 +1734,12 @@
         <v>87</v>
       </c>
       <c r="H14" s="1">
-        <v>45869</v>
+        <v>45862</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B15" t="s">
         <v>88</v>
@@ -1778,38 +1760,38 @@
         <v>93</v>
       </c>
       <c r="H15" s="1">
-        <v>45862</v>
+        <v>45829</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>15</v>
+        <v>94</v>
       </c>
       <c r="B16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C16" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D16" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E16" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F16" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G16" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H16" s="1">
-        <v>45829</v>
+        <v>45900</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>100</v>
+        <v>8</v>
       </c>
       <c r="B17" t="s">
         <v>101</v>
@@ -1830,7 +1812,7 @@
         <v>106</v>
       </c>
       <c r="H17" s="1">
-        <v>45900</v>
+        <v>45823</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
@@ -1856,38 +1838,38 @@
         <v>112</v>
       </c>
       <c r="H18" s="1">
-        <v>45823</v>
+        <v>45859</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>8</v>
+        <v>113</v>
       </c>
       <c r="B19" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C19" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D19" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F19" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G19" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H19" s="1">
-        <v>45859</v>
+        <v>45892</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>119</v>
+        <v>8</v>
       </c>
       <c r="B20" t="s">
         <v>120</v>
@@ -1908,12 +1890,12 @@
         <v>125</v>
       </c>
       <c r="H20" s="1">
-        <v>45892</v>
+        <v>45773</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B21" t="s">
         <v>126</v>
@@ -1931,36 +1913,36 @@
         <v>130</v>
       </c>
       <c r="G21" t="s">
-        <v>131</v>
+        <v>33</v>
       </c>
       <c r="H21" s="1">
-        <v>45773</v>
+        <v>45827</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B22" t="s">
+        <v>131</v>
+      </c>
+      <c r="C22" t="s">
         <v>132</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
         <v>133</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
         <v>134</v>
       </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
         <v>135</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>136</v>
       </c>
-      <c r="G22" t="s">
-        <v>39</v>
-      </c>
       <c r="H22" s="1">
-        <v>45827</v>
+        <v>45887</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
@@ -1986,12 +1968,12 @@
         <v>142</v>
       </c>
       <c r="H23" s="1">
-        <v>45887</v>
+        <v>45781</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B24" t="s">
         <v>143</v>
@@ -2012,12 +1994,12 @@
         <v>148</v>
       </c>
       <c r="H24" s="1">
-        <v>45781</v>
+        <v>45829</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B25" t="s">
         <v>149</v>
@@ -2038,12 +2020,12 @@
         <v>154</v>
       </c>
       <c r="H25" s="1">
-        <v>45829</v>
+        <v>45724</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B26" t="s">
         <v>155</v>
@@ -2064,38 +2046,38 @@
         <v>160</v>
       </c>
       <c r="H26" s="1">
-        <v>45724</v>
+        <v>45921</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>8</v>
+        <v>161</v>
       </c>
       <c r="B27" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C27" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D27" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E27" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F27" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G27" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H27" s="1">
-        <v>45921</v>
+        <v>45870</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>167</v>
+        <v>8</v>
       </c>
       <c r="B28" t="s">
         <v>168</v>
@@ -2116,7 +2098,7 @@
         <v>173</v>
       </c>
       <c r="H28" s="1">
-        <v>45870</v>
+        <v>45767</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
@@ -2142,12 +2124,12 @@
         <v>179</v>
       </c>
       <c r="H29" s="1">
-        <v>45767</v>
+        <v>45844</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B30" t="s">
         <v>180</v>
@@ -2168,12 +2150,12 @@
         <v>185</v>
       </c>
       <c r="H30" s="1">
-        <v>45844</v>
+        <v>45841</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B31" t="s">
         <v>186</v>
@@ -2194,12 +2176,12 @@
         <v>191</v>
       </c>
       <c r="H31" s="1">
-        <v>45841</v>
+        <v>45955</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B32" t="s">
         <v>192</v>
@@ -2220,41 +2202,41 @@
         <v>197</v>
       </c>
       <c r="H32" s="1">
-        <v>45955</v>
+        <v>45864</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B33" t="s">
+        <v>168</v>
+      </c>
+      <c r="C33" t="s">
         <v>198</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
         <v>199</v>
       </c>
-      <c r="D33" t="s">
+      <c r="E33" t="s">
         <v>200</v>
       </c>
-      <c r="E33" t="s">
+      <c r="F33" t="s">
         <v>201</v>
       </c>
-      <c r="F33" t="s">
+      <c r="G33" t="s">
         <v>202</v>
       </c>
-      <c r="G33" t="s">
-        <v>203</v>
-      </c>
       <c r="H33" s="1">
-        <v>45864</v>
+        <v>45801</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B34" t="s">
-        <v>174</v>
+        <v>203</v>
       </c>
       <c r="C34" t="s">
         <v>204</v>
@@ -2272,12 +2254,12 @@
         <v>208</v>
       </c>
       <c r="H34" s="1">
-        <v>45801</v>
+        <v>45815</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B35" t="s">
         <v>209</v>
@@ -2298,12 +2280,12 @@
         <v>214</v>
       </c>
       <c r="H35" s="1">
-        <v>45815</v>
+        <v>45773</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B36" t="s">
         <v>215</v>
@@ -2324,12 +2306,12 @@
         <v>220</v>
       </c>
       <c r="H36" s="1">
-        <v>45773</v>
+        <v>45871</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B37" t="s">
         <v>221</v>
@@ -2350,12 +2332,12 @@
         <v>226</v>
       </c>
       <c r="H37" s="1">
-        <v>45871</v>
+        <v>45886</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B38" t="s">
         <v>227</v>
@@ -2376,12 +2358,12 @@
         <v>232</v>
       </c>
       <c r="H38" s="1">
-        <v>45886</v>
+        <v>45781</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B39" t="s">
         <v>233</v>
@@ -2399,41 +2381,41 @@
         <v>237</v>
       </c>
       <c r="G39" t="s">
-        <v>238</v>
+        <v>154</v>
       </c>
       <c r="H39" s="1">
-        <v>45781</v>
+        <v>45821</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B40" t="s">
+        <v>238</v>
+      </c>
+      <c r="C40" t="s">
         <v>239</v>
       </c>
-      <c r="C40" t="s">
+      <c r="D40" t="s">
         <v>240</v>
       </c>
-      <c r="D40" t="s">
+      <c r="E40" t="s">
         <v>241</v>
       </c>
-      <c r="E40" t="s">
+      <c r="F40" t="s">
         <v>242</v>
       </c>
-      <c r="F40" t="s">
+      <c r="G40" t="s">
         <v>243</v>
       </c>
-      <c r="G40" t="s">
-        <v>160</v>
-      </c>
       <c r="H40" s="1">
-        <v>45821</v>
+        <v>45856</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B41" t="s">
         <v>244</v>
@@ -2454,12 +2436,12 @@
         <v>249</v>
       </c>
       <c r="H41" s="1">
-        <v>45856</v>
+        <v>45899</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B42" t="s">
         <v>250</v>
@@ -2480,12 +2462,12 @@
         <v>255</v>
       </c>
       <c r="H42" s="1">
-        <v>45899</v>
+        <v>45873</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B43" t="s">
         <v>256</v>
@@ -2506,12 +2488,12 @@
         <v>261</v>
       </c>
       <c r="H43" s="1">
-        <v>45873</v>
+        <v>45827</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B44" t="s">
         <v>262</v>
@@ -2532,12 +2514,12 @@
         <v>267</v>
       </c>
       <c r="H44" s="1">
-        <v>45827</v>
+        <v>45849</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B45" t="s">
         <v>268</v>
@@ -2558,7 +2540,7 @@
         <v>273</v>
       </c>
       <c r="H45" s="1">
-        <v>45849</v>
+        <v>45851</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
@@ -2584,7 +2566,7 @@
         <v>279</v>
       </c>
       <c r="H46" s="1">
-        <v>45851</v>
+        <v>45961</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
@@ -2610,7 +2592,7 @@
         <v>285</v>
       </c>
       <c r="H47" s="1">
-        <v>45961</v>
+        <v>45844</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
@@ -2636,7 +2618,7 @@
         <v>291</v>
       </c>
       <c r="H48" s="1">
-        <v>45844</v>
+        <v>45804</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
@@ -2662,32 +2644,6 @@
         <v>297</v>
       </c>
       <c r="H49" s="1">
-        <v>45804</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
-        <v>8</v>
-      </c>
-      <c r="B50" t="s">
-        <v>298</v>
-      </c>
-      <c r="C50" t="s">
-        <v>299</v>
-      </c>
-      <c r="D50" t="s">
-        <v>300</v>
-      </c>
-      <c r="E50" t="s">
-        <v>301</v>
-      </c>
-      <c r="F50" t="s">
-        <v>302</v>
-      </c>
-      <c r="G50" t="s">
-        <v>303</v>
-      </c>
-      <c r="H50" s="1">
         <v>45874</v>
       </c>
     </row>

</xml_diff>

<commit_message>
subir listados campaña corazul7
</commit_message>
<xml_diff>
--- a/campanas/260413_corazul/corazul_1_tuesday.xlsx
+++ b/campanas/260413_corazul/corazul_1_tuesday.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diegopaezmacias/GRIDDED.AGENCY local/00_GRIDDED AGENCY/cdn/campanas/260413_corazul/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A302FD52-50A0-9043-A6D2-012873BA9B3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7AEDDFC-4B48-3542-BC2E-2AAE675E6D02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="19560" windowHeight="24600" xr2:uid="{FE8E41CE-C1E5-794B-8212-B8E3CEE34DA9}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="campaña 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="DatosExternos_2" localSheetId="0" hidden="1">'campaña 1'!$A$1:$H$49</definedName>
+    <definedName name="DatosExternos_2" localSheetId="0" hidden="1">'campaña 1'!$A$1:$H$48</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="292">
   <si>
     <t>nombreNaviera</t>
   </si>
@@ -76,24 +76,6 @@
   </si>
   <si>
     <t>MSC Cruceros</t>
-  </si>
-  <si>
-    <t>Dolores</t>
-  </si>
-  <si>
-    <t>Vigara Dominguez</t>
-  </si>
-  <si>
-    <t>34691202094</t>
-  </si>
-  <si>
-    <t>lolivigara@hotmail.com</t>
-  </si>
-  <si>
-    <t>Entrepeñas N76 - portal D 5ºD</t>
-  </si>
-  <si>
-    <t>Madrid</t>
   </si>
   <si>
     <t>JUANA</t>
@@ -1045,8 +1027,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EBC5DAF2-265F-5C4B-9F14-50406A6420A0}" name="Ventas_Cuadruples_2025" displayName="Ventas_Cuadruples_2025" ref="A1:H49" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:H49" xr:uid="{7B6879F4-F5E9-40D9-A981-23B705F0A713}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EBC5DAF2-265F-5C4B-9F14-50406A6420A0}" name="Ventas_Cuadruples_2025" displayName="Ventas_Cuadruples_2025" ref="A1:H48" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:H48" xr:uid="{7B6879F4-F5E9-40D9-A981-23B705F0A713}"/>
   <tableColumns count="8">
     <tableColumn id="2" xr3:uid="{D7C59A67-56B1-FC40-A80E-0553C9334F80}" uniqueName="2" name="nombreNaviera" queryTableFieldId="2" dataDxfId="7"/>
     <tableColumn id="3" xr3:uid="{B6B681FD-4C35-654A-AEF6-F0A60C2EF737}" uniqueName="3" name="nombreCliente" queryTableFieldId="3" dataDxfId="6"/>
@@ -1358,7 +1340,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E88A72D-71A2-D844-BACB-214CA146513D}">
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
@@ -1401,7 +1383,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -1422,12 +1404,12 @@
         <v>15</v>
       </c>
       <c r="H2" s="1">
-        <v>45829</v>
+        <v>45837</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
         <v>16</v>
@@ -1448,12 +1430,12 @@
         <v>21</v>
       </c>
       <c r="H3" s="1">
-        <v>45837</v>
+        <v>45776</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4" t="s">
         <v>22</v>
@@ -1474,12 +1456,12 @@
         <v>27</v>
       </c>
       <c r="H4" s="1">
-        <v>45776</v>
+        <v>45793</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
         <v>28</v>
@@ -1500,7 +1482,7 @@
         <v>33</v>
       </c>
       <c r="H5" s="1">
-        <v>45793</v>
+        <v>45829</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -1526,7 +1508,7 @@
         <v>39</v>
       </c>
       <c r="H6" s="1">
-        <v>45829</v>
+        <v>45702</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -1552,7 +1534,7 @@
         <v>45</v>
       </c>
       <c r="H7" s="1">
-        <v>45702</v>
+        <v>45717</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
@@ -1578,12 +1560,12 @@
         <v>51</v>
       </c>
       <c r="H8" s="1">
-        <v>45717</v>
+        <v>45975</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" t="s">
         <v>52</v>
@@ -1604,12 +1586,12 @@
         <v>57</v>
       </c>
       <c r="H9" s="1">
-        <v>45975</v>
+        <v>45768</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
         <v>58</v>
@@ -1630,7 +1612,7 @@
         <v>63</v>
       </c>
       <c r="H10" s="1">
-        <v>45768</v>
+        <v>46013</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
@@ -1656,7 +1638,7 @@
         <v>69</v>
       </c>
       <c r="H11" s="1">
-        <v>46013</v>
+        <v>45722</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
@@ -1682,7 +1664,7 @@
         <v>75</v>
       </c>
       <c r="H12" s="1">
-        <v>45722</v>
+        <v>45869</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
@@ -1708,7 +1690,7 @@
         <v>81</v>
       </c>
       <c r="H13" s="1">
-        <v>45869</v>
+        <v>45862</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
@@ -1734,38 +1716,38 @@
         <v>87</v>
       </c>
       <c r="H14" s="1">
-        <v>45862</v>
+        <v>45829</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>9</v>
+        <v>88</v>
       </c>
       <c r="B15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C15" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D15" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E15" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F15" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G15" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H15" s="1">
-        <v>45829</v>
+        <v>45900</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>94</v>
+        <v>8</v>
       </c>
       <c r="B16" t="s">
         <v>95</v>
@@ -1786,7 +1768,7 @@
         <v>100</v>
       </c>
       <c r="H16" s="1">
-        <v>45900</v>
+        <v>45823</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
@@ -1812,38 +1794,38 @@
         <v>106</v>
       </c>
       <c r="H17" s="1">
-        <v>45823</v>
+        <v>45859</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>8</v>
+        <v>107</v>
       </c>
       <c r="B18" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C18" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D18" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E18" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F18" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G18" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H18" s="1">
-        <v>45859</v>
+        <v>45892</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>113</v>
+        <v>8</v>
       </c>
       <c r="B19" t="s">
         <v>114</v>
@@ -1864,12 +1846,12 @@
         <v>119</v>
       </c>
       <c r="H19" s="1">
-        <v>45892</v>
+        <v>45773</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B20" t="s">
         <v>120</v>
@@ -1887,36 +1869,36 @@
         <v>124</v>
       </c>
       <c r="G20" t="s">
-        <v>125</v>
+        <v>27</v>
       </c>
       <c r="H20" s="1">
-        <v>45773</v>
+        <v>45827</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B21" t="s">
+        <v>125</v>
+      </c>
+      <c r="C21" t="s">
         <v>126</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>127</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>128</v>
       </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>129</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>130</v>
       </c>
-      <c r="G21" t="s">
-        <v>33</v>
-      </c>
       <c r="H21" s="1">
-        <v>45827</v>
+        <v>45887</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
@@ -1942,12 +1924,12 @@
         <v>136</v>
       </c>
       <c r="H22" s="1">
-        <v>45887</v>
+        <v>45781</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B23" t="s">
         <v>137</v>
@@ -1968,7 +1950,7 @@
         <v>142</v>
       </c>
       <c r="H23" s="1">
-        <v>45781</v>
+        <v>45829</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
@@ -1994,12 +1976,12 @@
         <v>148</v>
       </c>
       <c r="H24" s="1">
-        <v>45829</v>
+        <v>45724</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B25" t="s">
         <v>149</v>
@@ -2020,38 +2002,38 @@
         <v>154</v>
       </c>
       <c r="H25" s="1">
-        <v>45724</v>
+        <v>45921</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>8</v>
+        <v>155</v>
       </c>
       <c r="B26" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C26" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D26" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E26" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F26" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G26" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H26" s="1">
-        <v>45921</v>
+        <v>45870</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>161</v>
+        <v>8</v>
       </c>
       <c r="B27" t="s">
         <v>162</v>
@@ -2072,7 +2054,7 @@
         <v>167</v>
       </c>
       <c r="H27" s="1">
-        <v>45870</v>
+        <v>45767</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
@@ -2098,12 +2080,12 @@
         <v>173</v>
       </c>
       <c r="H28" s="1">
-        <v>45767</v>
+        <v>45844</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B29" t="s">
         <v>174</v>
@@ -2124,12 +2106,12 @@
         <v>179</v>
       </c>
       <c r="H29" s="1">
-        <v>45844</v>
+        <v>45841</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B30" t="s">
         <v>180</v>
@@ -2150,12 +2132,12 @@
         <v>185</v>
       </c>
       <c r="H30" s="1">
-        <v>45841</v>
+        <v>45955</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B31" t="s">
         <v>186</v>
@@ -2176,7 +2158,7 @@
         <v>191</v>
       </c>
       <c r="H31" s="1">
-        <v>45955</v>
+        <v>45864</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
@@ -2184,25 +2166,25 @@
         <v>9</v>
       </c>
       <c r="B32" t="s">
+        <v>162</v>
+      </c>
+      <c r="C32" t="s">
         <v>192</v>
       </c>
-      <c r="C32" t="s">
+      <c r="D32" t="s">
         <v>193</v>
       </c>
-      <c r="D32" t="s">
+      <c r="E32" t="s">
         <v>194</v>
       </c>
-      <c r="E32" t="s">
+      <c r="F32" t="s">
         <v>195</v>
       </c>
-      <c r="F32" t="s">
+      <c r="G32" t="s">
         <v>196</v>
       </c>
-      <c r="G32" t="s">
-        <v>197</v>
-      </c>
       <c r="H32" s="1">
-        <v>45864</v>
+        <v>45801</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
@@ -2210,7 +2192,7 @@
         <v>9</v>
       </c>
       <c r="B33" t="s">
-        <v>168</v>
+        <v>197</v>
       </c>
       <c r="C33" t="s">
         <v>198</v>
@@ -2228,12 +2210,12 @@
         <v>202</v>
       </c>
       <c r="H33" s="1">
-        <v>45801</v>
+        <v>45815</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B34" t="s">
         <v>203</v>
@@ -2254,12 +2236,12 @@
         <v>208</v>
       </c>
       <c r="H34" s="1">
-        <v>45815</v>
+        <v>45773</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B35" t="s">
         <v>209</v>
@@ -2280,12 +2262,12 @@
         <v>214</v>
       </c>
       <c r="H35" s="1">
-        <v>45773</v>
+        <v>45871</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B36" t="s">
         <v>215</v>
@@ -2306,12 +2288,12 @@
         <v>220</v>
       </c>
       <c r="H36" s="1">
-        <v>45871</v>
+        <v>45886</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B37" t="s">
         <v>221</v>
@@ -2332,7 +2314,7 @@
         <v>226</v>
       </c>
       <c r="H37" s="1">
-        <v>45886</v>
+        <v>45781</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
@@ -2355,41 +2337,41 @@
         <v>231</v>
       </c>
       <c r="G38" t="s">
-        <v>232</v>
+        <v>148</v>
       </c>
       <c r="H38" s="1">
-        <v>45781</v>
+        <v>45821</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B39" t="s">
+        <v>232</v>
+      </c>
+      <c r="C39" t="s">
         <v>233</v>
       </c>
-      <c r="C39" t="s">
+      <c r="D39" t="s">
         <v>234</v>
       </c>
-      <c r="D39" t="s">
+      <c r="E39" t="s">
         <v>235</v>
       </c>
-      <c r="E39" t="s">
+      <c r="F39" t="s">
         <v>236</v>
       </c>
-      <c r="F39" t="s">
+      <c r="G39" t="s">
         <v>237</v>
       </c>
-      <c r="G39" t="s">
-        <v>154</v>
-      </c>
       <c r="H39" s="1">
-        <v>45821</v>
+        <v>45856</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B40" t="s">
         <v>238</v>
@@ -2410,12 +2392,12 @@
         <v>243</v>
       </c>
       <c r="H40" s="1">
-        <v>45856</v>
+        <v>45899</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B41" t="s">
         <v>244</v>
@@ -2436,12 +2418,12 @@
         <v>249</v>
       </c>
       <c r="H41" s="1">
-        <v>45899</v>
+        <v>45873</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B42" t="s">
         <v>250</v>
@@ -2462,7 +2444,7 @@
         <v>255</v>
       </c>
       <c r="H42" s="1">
-        <v>45873</v>
+        <v>45827</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
@@ -2488,12 +2470,12 @@
         <v>261</v>
       </c>
       <c r="H43" s="1">
-        <v>45827</v>
+        <v>45849</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B44" t="s">
         <v>262</v>
@@ -2514,7 +2496,7 @@
         <v>267</v>
       </c>
       <c r="H44" s="1">
-        <v>45849</v>
+        <v>45851</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
@@ -2540,7 +2522,7 @@
         <v>273</v>
       </c>
       <c r="H45" s="1">
-        <v>45851</v>
+        <v>45961</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
@@ -2566,7 +2548,7 @@
         <v>279</v>
       </c>
       <c r="H46" s="1">
-        <v>45961</v>
+        <v>45844</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
@@ -2592,7 +2574,7 @@
         <v>285</v>
       </c>
       <c r="H47" s="1">
-        <v>45844</v>
+        <v>45804</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
@@ -2618,32 +2600,6 @@
         <v>291</v>
       </c>
       <c r="H48" s="1">
-        <v>45804</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>8</v>
-      </c>
-      <c r="B49" t="s">
-        <v>292</v>
-      </c>
-      <c r="C49" t="s">
-        <v>293</v>
-      </c>
-      <c r="D49" t="s">
-        <v>294</v>
-      </c>
-      <c r="E49" t="s">
-        <v>295</v>
-      </c>
-      <c r="F49" t="s">
-        <v>296</v>
-      </c>
-      <c r="G49" t="s">
-        <v>297</v>
-      </c>
-      <c r="H49" s="1">
         <v>45874</v>
       </c>
     </row>

</xml_diff>

<commit_message>
subir listados campaña corazul8
</commit_message>
<xml_diff>
--- a/campanas/260413_corazul/corazul_1_tuesday.xlsx
+++ b/campanas/260413_corazul/corazul_1_tuesday.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diegopaezmacias/GRIDDED.AGENCY local/00_GRIDDED AGENCY/cdn/campanas/260413_corazul/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7AEDDFC-4B48-3542-BC2E-2AAE675E6D02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B29E9C1-EFAA-1543-88E9-ADF87E9EEC63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="19560" windowHeight="24600" xr2:uid="{FE8E41CE-C1E5-794B-8212-B8E3CEE34DA9}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="campaña 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="DatosExternos_2" localSheetId="0" hidden="1">'campaña 1'!$A$1:$H$48</definedName>
+    <definedName name="DatosExternos_2" localSheetId="0" hidden="1">'campaña 1'!$A$1:$H$47</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="286">
   <si>
     <t>nombreNaviera</t>
   </si>
@@ -76,24 +76,6 @@
   </si>
   <si>
     <t>MSC Cruceros</t>
-  </si>
-  <si>
-    <t>JUANA</t>
-  </si>
-  <si>
-    <t>LÓPEZ LÓPEZ</t>
-  </si>
-  <si>
-    <t>600245838</t>
-  </si>
-  <si>
-    <t>julop888@gmail.com</t>
-  </si>
-  <si>
-    <t>CALLE DOCTOR FLEMING</t>
-  </si>
-  <si>
-    <t>OGIJARES</t>
   </si>
   <si>
     <t xml:space="preserve">CORINA </t>
@@ -1027,8 +1009,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EBC5DAF2-265F-5C4B-9F14-50406A6420A0}" name="Ventas_Cuadruples_2025" displayName="Ventas_Cuadruples_2025" ref="A1:H48" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:H48" xr:uid="{7B6879F4-F5E9-40D9-A981-23B705F0A713}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EBC5DAF2-265F-5C4B-9F14-50406A6420A0}" name="Ventas_Cuadruples_2025" displayName="Ventas_Cuadruples_2025" ref="A1:H47" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:H47" xr:uid="{7B6879F4-F5E9-40D9-A981-23B705F0A713}"/>
   <tableColumns count="8">
     <tableColumn id="2" xr3:uid="{D7C59A67-56B1-FC40-A80E-0553C9334F80}" uniqueName="2" name="nombreNaviera" queryTableFieldId="2" dataDxfId="7"/>
     <tableColumn id="3" xr3:uid="{B6B681FD-4C35-654A-AEF6-F0A60C2EF737}" uniqueName="3" name="nombreCliente" queryTableFieldId="3" dataDxfId="6"/>
@@ -1340,7 +1322,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E88A72D-71A2-D844-BACB-214CA146513D}">
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
@@ -1383,7 +1365,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -1404,12 +1386,12 @@
         <v>15</v>
       </c>
       <c r="H2" s="1">
-        <v>45837</v>
+        <v>45776</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
         <v>16</v>
@@ -1430,12 +1412,12 @@
         <v>21</v>
       </c>
       <c r="H3" s="1">
-        <v>45776</v>
+        <v>45793</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
         <v>22</v>
@@ -1456,7 +1438,7 @@
         <v>27</v>
       </c>
       <c r="H4" s="1">
-        <v>45793</v>
+        <v>45829</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
@@ -1482,7 +1464,7 @@
         <v>33</v>
       </c>
       <c r="H5" s="1">
-        <v>45829</v>
+        <v>45702</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -1508,7 +1490,7 @@
         <v>39</v>
       </c>
       <c r="H6" s="1">
-        <v>45702</v>
+        <v>45717</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -1534,12 +1516,12 @@
         <v>45</v>
       </c>
       <c r="H7" s="1">
-        <v>45717</v>
+        <v>45975</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
         <v>46</v>
@@ -1560,12 +1542,12 @@
         <v>51</v>
       </c>
       <c r="H8" s="1">
-        <v>45975</v>
+        <v>45768</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B9" t="s">
         <v>52</v>
@@ -1586,7 +1568,7 @@
         <v>57</v>
       </c>
       <c r="H9" s="1">
-        <v>45768</v>
+        <v>46013</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
@@ -1612,7 +1594,7 @@
         <v>63</v>
       </c>
       <c r="H10" s="1">
-        <v>46013</v>
+        <v>45722</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
@@ -1638,7 +1620,7 @@
         <v>69</v>
       </c>
       <c r="H11" s="1">
-        <v>45722</v>
+        <v>45869</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
@@ -1664,7 +1646,7 @@
         <v>75</v>
       </c>
       <c r="H12" s="1">
-        <v>45869</v>
+        <v>45862</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
@@ -1690,38 +1672,38 @@
         <v>81</v>
       </c>
       <c r="H13" s="1">
-        <v>45862</v>
+        <v>45829</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>9</v>
+        <v>82</v>
       </c>
       <c r="B14" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C14" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D14" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E14" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H14" s="1">
-        <v>45829</v>
+        <v>45900</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>88</v>
+        <v>8</v>
       </c>
       <c r="B15" t="s">
         <v>89</v>
@@ -1742,7 +1724,7 @@
         <v>94</v>
       </c>
       <c r="H15" s="1">
-        <v>45900</v>
+        <v>45823</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
@@ -1768,38 +1750,38 @@
         <v>100</v>
       </c>
       <c r="H16" s="1">
-        <v>45823</v>
+        <v>45859</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>8</v>
+        <v>101</v>
       </c>
       <c r="B17" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C17" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D17" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E17" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F17" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G17" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H17" s="1">
-        <v>45859</v>
+        <v>45892</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>107</v>
+        <v>8</v>
       </c>
       <c r="B18" t="s">
         <v>108</v>
@@ -1820,12 +1802,12 @@
         <v>113</v>
       </c>
       <c r="H18" s="1">
-        <v>45892</v>
+        <v>45773</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B19" t="s">
         <v>114</v>
@@ -1843,36 +1825,36 @@
         <v>118</v>
       </c>
       <c r="G19" t="s">
-        <v>119</v>
+        <v>21</v>
       </c>
       <c r="H19" s="1">
-        <v>45773</v>
+        <v>45827</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C20" t="s">
         <v>120</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>121</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>122</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
         <v>123</v>
       </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
         <v>124</v>
       </c>
-      <c r="G20" t="s">
-        <v>27</v>
-      </c>
       <c r="H20" s="1">
-        <v>45827</v>
+        <v>45887</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
@@ -1898,12 +1880,12 @@
         <v>130</v>
       </c>
       <c r="H21" s="1">
-        <v>45887</v>
+        <v>45781</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B22" t="s">
         <v>131</v>
@@ -1924,7 +1906,7 @@
         <v>136</v>
       </c>
       <c r="H22" s="1">
-        <v>45781</v>
+        <v>45829</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
@@ -1950,12 +1932,12 @@
         <v>142</v>
       </c>
       <c r="H23" s="1">
-        <v>45829</v>
+        <v>45724</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B24" t="s">
         <v>143</v>
@@ -1976,38 +1958,38 @@
         <v>148</v>
       </c>
       <c r="H24" s="1">
-        <v>45724</v>
+        <v>45921</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>8</v>
+        <v>149</v>
       </c>
       <c r="B25" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C25" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D25" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E25" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F25" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G25" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H25" s="1">
-        <v>45921</v>
+        <v>45870</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>155</v>
+        <v>8</v>
       </c>
       <c r="B26" t="s">
         <v>156</v>
@@ -2028,7 +2010,7 @@
         <v>161</v>
       </c>
       <c r="H26" s="1">
-        <v>45870</v>
+        <v>45767</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
@@ -2054,12 +2036,12 @@
         <v>167</v>
       </c>
       <c r="H27" s="1">
-        <v>45767</v>
+        <v>45844</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B28" t="s">
         <v>168</v>
@@ -2080,12 +2062,12 @@
         <v>173</v>
       </c>
       <c r="H28" s="1">
-        <v>45844</v>
+        <v>45841</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B29" t="s">
         <v>174</v>
@@ -2106,12 +2088,12 @@
         <v>179</v>
       </c>
       <c r="H29" s="1">
-        <v>45841</v>
+        <v>45955</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B30" t="s">
         <v>180</v>
@@ -2132,7 +2114,7 @@
         <v>185</v>
       </c>
       <c r="H30" s="1">
-        <v>45955</v>
+        <v>45864</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
@@ -2140,25 +2122,25 @@
         <v>9</v>
       </c>
       <c r="B31" t="s">
+        <v>156</v>
+      </c>
+      <c r="C31" t="s">
         <v>186</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>187</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>188</v>
       </c>
-      <c r="E31" t="s">
+      <c r="F31" t="s">
         <v>189</v>
       </c>
-      <c r="F31" t="s">
+      <c r="G31" t="s">
         <v>190</v>
       </c>
-      <c r="G31" t="s">
-        <v>191</v>
-      </c>
       <c r="H31" s="1">
-        <v>45864</v>
+        <v>45801</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
@@ -2166,7 +2148,7 @@
         <v>9</v>
       </c>
       <c r="B32" t="s">
-        <v>162</v>
+        <v>191</v>
       </c>
       <c r="C32" t="s">
         <v>192</v>
@@ -2184,12 +2166,12 @@
         <v>196</v>
       </c>
       <c r="H32" s="1">
-        <v>45801</v>
+        <v>45815</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B33" t="s">
         <v>197</v>
@@ -2210,12 +2192,12 @@
         <v>202</v>
       </c>
       <c r="H33" s="1">
-        <v>45815</v>
+        <v>45773</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B34" t="s">
         <v>203</v>
@@ -2236,12 +2218,12 @@
         <v>208</v>
       </c>
       <c r="H34" s="1">
-        <v>45773</v>
+        <v>45871</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B35" t="s">
         <v>209</v>
@@ -2262,12 +2244,12 @@
         <v>214</v>
       </c>
       <c r="H35" s="1">
-        <v>45871</v>
+        <v>45886</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B36" t="s">
         <v>215</v>
@@ -2288,7 +2270,7 @@
         <v>220</v>
       </c>
       <c r="H36" s="1">
-        <v>45886</v>
+        <v>45781</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
@@ -2311,41 +2293,41 @@
         <v>225</v>
       </c>
       <c r="G37" t="s">
-        <v>226</v>
+        <v>142</v>
       </c>
       <c r="H37" s="1">
-        <v>45781</v>
+        <v>45821</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B38" t="s">
+        <v>226</v>
+      </c>
+      <c r="C38" t="s">
         <v>227</v>
       </c>
-      <c r="C38" t="s">
+      <c r="D38" t="s">
         <v>228</v>
       </c>
-      <c r="D38" t="s">
+      <c r="E38" t="s">
         <v>229</v>
       </c>
-      <c r="E38" t="s">
+      <c r="F38" t="s">
         <v>230</v>
       </c>
-      <c r="F38" t="s">
+      <c r="G38" t="s">
         <v>231</v>
       </c>
-      <c r="G38" t="s">
-        <v>148</v>
-      </c>
       <c r="H38" s="1">
-        <v>45821</v>
+        <v>45856</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B39" t="s">
         <v>232</v>
@@ -2366,12 +2348,12 @@
         <v>237</v>
       </c>
       <c r="H39" s="1">
-        <v>45856</v>
+        <v>45899</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B40" t="s">
         <v>238</v>
@@ -2392,12 +2374,12 @@
         <v>243</v>
       </c>
       <c r="H40" s="1">
-        <v>45899</v>
+        <v>45873</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B41" t="s">
         <v>244</v>
@@ -2418,7 +2400,7 @@
         <v>249</v>
       </c>
       <c r="H41" s="1">
-        <v>45873</v>
+        <v>45827</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
@@ -2444,12 +2426,12 @@
         <v>255</v>
       </c>
       <c r="H42" s="1">
-        <v>45827</v>
+        <v>45849</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B43" t="s">
         <v>256</v>
@@ -2470,7 +2452,7 @@
         <v>261</v>
       </c>
       <c r="H43" s="1">
-        <v>45849</v>
+        <v>45851</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
@@ -2496,7 +2478,7 @@
         <v>267</v>
       </c>
       <c r="H44" s="1">
-        <v>45851</v>
+        <v>45961</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
@@ -2522,7 +2504,7 @@
         <v>273</v>
       </c>
       <c r="H45" s="1">
-        <v>45961</v>
+        <v>45844</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
@@ -2548,7 +2530,7 @@
         <v>279</v>
       </c>
       <c r="H46" s="1">
-        <v>45844</v>
+        <v>45804</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
@@ -2574,32 +2556,6 @@
         <v>285</v>
       </c>
       <c r="H47" s="1">
-        <v>45804</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
-        <v>8</v>
-      </c>
-      <c r="B48" t="s">
-        <v>286</v>
-      </c>
-      <c r="C48" t="s">
-        <v>287</v>
-      </c>
-      <c r="D48" t="s">
-        <v>288</v>
-      </c>
-      <c r="E48" t="s">
-        <v>289</v>
-      </c>
-      <c r="F48" t="s">
-        <v>290</v>
-      </c>
-      <c r="G48" t="s">
-        <v>291</v>
-      </c>
-      <c r="H48" s="1">
         <v>45874</v>
       </c>
     </row>

</xml_diff>